<commit_message>
Update full database from Kas_Bendahara_Kelas_5A_2026-2027 Update.xlsx (Rp 3.660.000, 183 lunas) and add real-time search on Payments and Students tabs
</commit_message>
<xml_diff>
--- a/public/Kas_Bendahara_Kelas5A_SDS-KasihAnanda_TA2026-2027.xlsx
+++ b/public/Kas_Bendahara_Kelas5A_SDS-KasihAnanda_TA2026-2027.xlsx
@@ -1,42 +1,314 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Indah 2025\Project Indah\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3A351502-C7E1-4416-B521-A53D368F741A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="23880" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Pembayaran Kas 12 Bulan" sheetId="1" r:id="rId1"/>
     <sheet name="Pengeluaran Kas" sheetId="2" r:id="rId2"/>
   </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="90">
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Nama Siswa</t>
+  </si>
+  <si>
+    <t>No. HP / WA</t>
+  </si>
+  <si>
+    <t>Juli 2026</t>
+  </si>
+  <si>
+    <t>Agustus 2026</t>
+  </si>
+  <si>
+    <t>September 2026</t>
+  </si>
+  <si>
+    <t>Oktober 2026</t>
+  </si>
+  <si>
+    <t>November 2026</t>
+  </si>
+  <si>
+    <t>Desember 2026</t>
+  </si>
+  <si>
+    <t>Januari 2027</t>
+  </si>
+  <si>
+    <t>Februari 2027</t>
+  </si>
+  <si>
+    <t>Maret 2027</t>
+  </si>
+  <si>
+    <t>April 2027</t>
+  </si>
+  <si>
+    <t>Mei 2027</t>
+  </si>
+  <si>
+    <t>Juni 2027</t>
+  </si>
+  <si>
+    <t>Total Lunas</t>
+  </si>
+  <si>
+    <t>Total Nominal (Rp)</t>
+  </si>
+  <si>
+    <t>Adiara Zahwa Aprella</t>
+  </si>
+  <si>
+    <t>082125470951</t>
+  </si>
+  <si>
+    <t>2/12</t>
+  </si>
+  <si>
+    <t>Alesha Fitria Khairunnisa</t>
+  </si>
+  <si>
+    <t>081281920272</t>
+  </si>
+  <si>
+    <t>6/12</t>
+  </si>
+  <si>
+    <t>Alicia Alverina Carter</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Allesya Alvera Meina Lengkong</t>
+  </si>
+  <si>
+    <t>0/12</t>
+  </si>
+  <si>
+    <t>Allysia Leilanie Yasmine</t>
+  </si>
+  <si>
+    <t>Ar Kenzie Kiaka Putra</t>
+  </si>
+  <si>
+    <t>Cathy Charissa Hutauruk</t>
+  </si>
+  <si>
+    <t>Cavello Vincenzo Pratama</t>
+  </si>
+  <si>
+    <t>082130355514</t>
+  </si>
+  <si>
+    <t>12/12</t>
+  </si>
+  <si>
+    <t>Chelsea Vebian</t>
+  </si>
+  <si>
+    <t>087894587966</t>
+  </si>
+  <si>
+    <t>Cleo Vennya Donita</t>
+  </si>
+  <si>
+    <t>08111742629</t>
+  </si>
+  <si>
+    <t>3/12</t>
+  </si>
+  <si>
+    <t>Cleona Uli Malau</t>
+  </si>
+  <si>
+    <t>Cleva Anastasya Tanjung</t>
+  </si>
+  <si>
+    <t>Darrell Gavriel Oliver</t>
+  </si>
+  <si>
+    <t>5/12</t>
+  </si>
+  <si>
+    <t>Diandra Sapta Pratama</t>
+  </si>
+  <si>
+    <t>Fahira Anindita Nurhakim</t>
+  </si>
+  <si>
+    <t>Fazila Azzahra</t>
+  </si>
+  <si>
+    <t>Fransisca</t>
+  </si>
+  <si>
+    <t>Josua Hamonangan Slahaan</t>
+  </si>
+  <si>
+    <t>Jusuf Habibi Muchtar</t>
+  </si>
+  <si>
+    <t>Khaerul Basyar Rukmana</t>
+  </si>
+  <si>
+    <t>085710401552</t>
+  </si>
+  <si>
+    <t>Khairunnisa Dwi Kurniawan</t>
+  </si>
+  <si>
+    <t>Kim Reynand Andah Pranaja</t>
+  </si>
+  <si>
+    <t>085117070159</t>
+  </si>
+  <si>
+    <t>Lutfi Khoirul Nur Ramadhan</t>
+  </si>
+  <si>
+    <t>081283016613</t>
+  </si>
+  <si>
+    <t>Marco Alejandro Mendoza Retno</t>
+  </si>
+  <si>
+    <t>081808251119</t>
+  </si>
+  <si>
+    <t>Maryam Audra Milly</t>
+  </si>
+  <si>
+    <t>085176651200</t>
+  </si>
+  <si>
+    <t>Muhammad Danish Ali Haidari</t>
+  </si>
+  <si>
+    <t>Muhammad Raja El Firdaus</t>
+  </si>
+  <si>
+    <t>087745525749</t>
+  </si>
+  <si>
+    <t>Muhammad Rifat Ramadhan</t>
+  </si>
+  <si>
+    <t>081212855837</t>
+  </si>
+  <si>
+    <t>Muhammad Zlatan Alkhalifi</t>
+  </si>
+  <si>
+    <t>081216100160</t>
+  </si>
+  <si>
+    <t>Nathaniel Raphael</t>
+  </si>
+  <si>
+    <t>Naura Alvy Zahya</t>
+  </si>
+  <si>
+    <t>081291890142</t>
+  </si>
+  <si>
+    <t>Queenzha Aqila</t>
+  </si>
+  <si>
+    <t>081288071004</t>
+  </si>
+  <si>
+    <t>Satya Akbar Putra</t>
+  </si>
+  <si>
+    <t>Syafhia Nazruliza</t>
+  </si>
+  <si>
+    <t>Viola Callista Donita</t>
+  </si>
+  <si>
+    <t>Tanggal</t>
+  </si>
+  <si>
+    <t>Kategori</t>
+  </si>
+  <si>
+    <t>Uraian Keperluan</t>
+  </si>
+  <si>
+    <t>Nominal (Rp)</t>
+  </si>
+  <si>
+    <t>2026-08-04</t>
+  </si>
+  <si>
+    <t>Lain-lain</t>
+  </si>
+  <si>
+    <t>Tissue 2 Ply A Basics 600gram 2pcs</t>
+  </si>
+  <si>
+    <t>Stella Aerosol Balinese Jasmine Sensation Pengharum Ruangan 350ml 2pcs</t>
+  </si>
+  <si>
+    <t>2026-07-31</t>
+  </si>
+  <si>
+    <t>Air galon 2 @22000</t>
+  </si>
+  <si>
+    <t>Tisue</t>
+  </si>
+  <si>
+    <t>Fotokopi &amp; Cetak Soal</t>
+  </si>
+  <si>
+    <t>FC jadwal 35 @500</t>
+  </si>
+  <si>
+    <t>LKPD MPLS 20 @500</t>
+  </si>
+  <si>
+    <t>LKPD Wali kelas 35 @500</t>
+  </si>
+  <si>
+    <t>Jenguk mama Danish</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -65,14 +337,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -397,71 +678,78 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q36"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:R37"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="27.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.25" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>No</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Nama Siswa</v>
-      </c>
-      <c r="C1" t="str">
-        <v>No. HP / WA</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Juli 2026</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Agustus 2026</v>
-      </c>
-      <c r="F1" t="str">
-        <v>September 2026</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Oktober 2026</v>
-      </c>
-      <c r="H1" t="str">
-        <v>November 2026</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Desember 2026</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Januari 2027</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Februari 2027</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Maret 2027</v>
-      </c>
-      <c r="M1" t="str">
-        <v>April 2027</v>
-      </c>
-      <c r="N1" t="str">
-        <v>Mei 2027</v>
-      </c>
-      <c r="O1" t="str">
-        <v>Juni 2027</v>
-      </c>
-      <c r="P1" t="str">
-        <v>Total Lunas</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>Total Nominal (Rp)</v>
-      </c>
-    </row>
-    <row r="2">
+    <row r="1" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="str">
-        <v>Adiara Zahwa Aprella</v>
-      </c>
-      <c r="C2" t="str">
-        <v>082125470951</v>
+      <c r="B2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
       </c>
       <c r="D2">
         <v>20000</v>
@@ -499,22 +787,23 @@
       <c r="O2">
         <v>0</v>
       </c>
-      <c r="P2" t="str">
-        <v>2/12</v>
+      <c r="P2" t="s">
+        <v>19</v>
       </c>
       <c r="Q2">
+        <f>SUM(D2:O2)</f>
         <v>40000</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="str">
-        <v>Alesha Fitria Khairunnisa</v>
-      </c>
-      <c r="C3" t="str">
-        <v>081281920272</v>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
       </c>
       <c r="D3">
         <v>20000</v>
@@ -552,22 +841,23 @@
       <c r="O3">
         <v>0</v>
       </c>
-      <c r="P3" t="str">
-        <v>6/12</v>
+      <c r="P3" t="s">
+        <v>22</v>
       </c>
       <c r="Q3">
+        <f t="shared" ref="Q3:Q36" si="0">SUM(D3:O3)</f>
         <v>120000</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" t="str">
-        <v>Alicia Alverina Carter</v>
-      </c>
-      <c r="C4" t="str">
-        <v>-</v>
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
+        <v>24</v>
       </c>
       <c r="D4">
         <v>20000</v>
@@ -605,75 +895,77 @@
       <c r="O4">
         <v>0</v>
       </c>
-      <c r="P4" t="str">
-        <v>6/12</v>
+      <c r="P4" t="s">
+        <v>22</v>
       </c>
       <c r="Q4">
+        <f t="shared" si="0"/>
         <v>120000</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" t="str">
-        <v>Allesya Alvera Meina Lengkong</v>
-      </c>
-      <c r="C5" t="str">
-        <v>-</v>
+      <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" t="s">
+        <v>24</v>
       </c>
       <c r="D5">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="E5">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="F5">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="H5">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="I5">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="J5">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="K5">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="L5">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="M5">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="N5">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="O5">
-        <v>20000</v>
-      </c>
-      <c r="P5" t="str">
-        <v>12/12</v>
+        <v>0</v>
+      </c>
+      <c r="P5" t="s">
+        <v>26</v>
       </c>
       <c r="Q5">
-        <v>240000</v>
-      </c>
-    </row>
-    <row r="6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" t="str">
-        <v>Allysia Leilanie Yasmine</v>
-      </c>
-      <c r="C6" t="str">
-        <v>-</v>
+      <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" t="s">
+        <v>24</v>
       </c>
       <c r="D6">
         <v>20000</v>
@@ -691,7 +983,7 @@
         <v>20000</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="J6">
         <v>0</v>
@@ -711,37 +1003,41 @@
       <c r="O6">
         <v>0</v>
       </c>
-      <c r="P6" t="str">
-        <v>5/12</v>
+      <c r="P6" t="s">
+        <v>26</v>
       </c>
       <c r="Q6">
-        <v>100000</v>
-      </c>
-    </row>
-    <row r="7">
+        <f t="shared" si="0"/>
+        <v>120000</v>
+      </c>
+      <c r="R6" s="1">
+        <v>46252</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" t="str">
-        <v>Ar Kenzie Kiaka Putra</v>
-      </c>
-      <c r="C7" t="str">
-        <v>-</v>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>24</v>
       </c>
       <c r="D7">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="E7">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="F7">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="I7">
         <v>0</v>
@@ -764,22 +1060,23 @@
       <c r="O7">
         <v>0</v>
       </c>
-      <c r="P7" t="str">
-        <v>5/12</v>
+      <c r="P7" t="s">
+        <v>26</v>
       </c>
       <c r="Q7">
-        <v>100000</v>
-      </c>
-    </row>
-    <row r="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" t="str">
-        <v>Cathy Charissa Hutauruk</v>
-      </c>
-      <c r="C8" t="str">
-        <v>-</v>
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" t="s">
+        <v>24</v>
       </c>
       <c r="D8">
         <v>20000</v>
@@ -791,10 +1088,10 @@
         <v>20000</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="I8">
         <v>0</v>
@@ -817,22 +1114,26 @@
       <c r="O8">
         <v>0</v>
       </c>
-      <c r="P8" t="str">
-        <v>3/12</v>
+      <c r="P8" t="s">
+        <v>26</v>
       </c>
       <c r="Q8">
-        <v>60000</v>
-      </c>
-    </row>
-    <row r="9">
+        <f t="shared" si="0"/>
+        <v>100000</v>
+      </c>
+      <c r="R8" s="1">
+        <v>46184</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" t="str">
-        <v>Cavello Vincenzo Pratama</v>
-      </c>
-      <c r="C9" t="str">
-        <v>082130355514</v>
+      <c r="B9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" t="s">
+        <v>31</v>
       </c>
       <c r="D9">
         <v>20000</v>
@@ -870,22 +1171,23 @@
       <c r="O9">
         <v>20000</v>
       </c>
-      <c r="P9" t="str">
-        <v>12/12</v>
+      <c r="P9" t="s">
+        <v>32</v>
       </c>
       <c r="Q9">
+        <f t="shared" si="0"/>
         <v>240000</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10" t="str">
-        <v>Chelsea Vebian</v>
-      </c>
-      <c r="C10" t="str">
-        <v>087894587966</v>
+      <c r="B10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" t="s">
+        <v>34</v>
       </c>
       <c r="D10">
         <v>20000</v>
@@ -923,22 +1225,23 @@
       <c r="O10">
         <v>20000</v>
       </c>
-      <c r="P10" t="str">
-        <v>12/12</v>
+      <c r="P10" t="s">
+        <v>32</v>
       </c>
       <c r="Q10">
+        <f t="shared" si="0"/>
         <v>240000</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11" t="str">
-        <v>Cleo Vennya Donita</v>
-      </c>
-      <c r="C11" t="str">
-        <v>08111742629</v>
+      <c r="B11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" t="s">
+        <v>36</v>
       </c>
       <c r="D11">
         <v>20000</v>
@@ -976,37 +1279,38 @@
       <c r="O11">
         <v>0</v>
       </c>
-      <c r="P11" t="str">
-        <v>3/12</v>
+      <c r="P11" t="s">
+        <v>37</v>
       </c>
       <c r="Q11">
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12" t="str">
-        <v>Cleona Uli Malau</v>
-      </c>
-      <c r="C12" t="str">
-        <v>-</v>
+      <c r="B12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" t="s">
+        <v>24</v>
       </c>
       <c r="D12">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="H12">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="I12">
         <v>0</v>
@@ -1029,37 +1333,38 @@
       <c r="O12">
         <v>0</v>
       </c>
-      <c r="P12" t="str">
-        <v>0/12</v>
+      <c r="P12" t="s">
+        <v>26</v>
       </c>
       <c r="Q12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
+        <f t="shared" si="0"/>
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13" t="str">
-        <v>Cleva Anastasya Tanjung</v>
-      </c>
-      <c r="C13" t="str">
-        <v>-</v>
+      <c r="B13" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" t="s">
+        <v>24</v>
       </c>
       <c r="D13">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="E13">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="H13">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="I13">
         <v>0</v>
@@ -1082,22 +1387,26 @@
       <c r="O13">
         <v>0</v>
       </c>
-      <c r="P13" t="str">
-        <v>0/12</v>
+      <c r="P13" t="s">
+        <v>26</v>
       </c>
       <c r="Q13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
+        <f t="shared" si="0"/>
+        <v>100000</v>
+      </c>
+      <c r="R13" s="1">
+        <v>46258</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
-      <c r="B14" t="str">
-        <v>Darrell Gavriel Oliver</v>
-      </c>
-      <c r="C14" t="str">
-        <v>-</v>
+      <c r="B14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" t="s">
+        <v>24</v>
       </c>
       <c r="D14">
         <v>20000</v>
@@ -1135,22 +1444,23 @@
       <c r="O14">
         <v>0</v>
       </c>
-      <c r="P14" t="str">
-        <v>5/12</v>
+      <c r="P14" t="s">
+        <v>41</v>
       </c>
       <c r="Q14">
+        <f t="shared" si="0"/>
         <v>100000</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
-      <c r="B15" t="str">
-        <v>Diandra Sapta Pratama</v>
-      </c>
-      <c r="C15" t="str">
-        <v>-</v>
+      <c r="B15" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" t="s">
+        <v>24</v>
       </c>
       <c r="D15">
         <v>20000</v>
@@ -1188,22 +1498,23 @@
       <c r="O15">
         <v>0</v>
       </c>
-      <c r="P15" t="str">
-        <v>6/12</v>
+      <c r="P15" t="s">
+        <v>22</v>
       </c>
       <c r="Q15">
+        <f t="shared" si="0"/>
         <v>120000</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
-      <c r="B16" t="str">
-        <v>Fahira Anindita Nurhakim</v>
-      </c>
-      <c r="C16" t="str">
-        <v>-</v>
+      <c r="B16" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" t="s">
+        <v>24</v>
       </c>
       <c r="D16">
         <v>20000</v>
@@ -1241,28 +1552,29 @@
       <c r="O16">
         <v>20000</v>
       </c>
-      <c r="P16" t="str">
-        <v>12/12</v>
+      <c r="P16" t="s">
+        <v>32</v>
       </c>
       <c r="Q16">
+        <f t="shared" si="0"/>
         <v>240000</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
-      <c r="B17" t="str">
-        <v>Fazila Azzahra</v>
-      </c>
-      <c r="C17" t="str">
-        <v>-</v>
+      <c r="B17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" t="s">
+        <v>24</v>
       </c>
       <c r="D17">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="E17">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="F17">
         <v>0</v>
@@ -1294,22 +1606,26 @@
       <c r="O17">
         <v>0</v>
       </c>
-      <c r="P17" t="str">
-        <v>0/12</v>
+      <c r="P17" t="s">
+        <v>26</v>
       </c>
       <c r="Q17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
+        <f t="shared" si="0"/>
+        <v>40000</v>
+      </c>
+      <c r="R17" s="1">
+        <v>46240</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
-      <c r="B18" t="str">
-        <v>Fransisca</v>
-      </c>
-      <c r="C18" t="str">
-        <v>-</v>
+      <c r="B18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" t="s">
+        <v>24</v>
       </c>
       <c r="D18">
         <v>0</v>
@@ -1347,22 +1663,23 @@
       <c r="O18">
         <v>0</v>
       </c>
-      <c r="P18" t="str">
-        <v>0/12</v>
+      <c r="P18" t="s">
+        <v>26</v>
       </c>
       <c r="Q18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
-      <c r="B19" t="str">
-        <v>Josua Hamonangan Slahaan</v>
-      </c>
-      <c r="C19" t="str">
-        <v>-</v>
+      <c r="B19" t="s">
+        <v>46</v>
+      </c>
+      <c r="C19" t="s">
+        <v>24</v>
       </c>
       <c r="D19">
         <v>20000</v>
@@ -1400,22 +1717,23 @@
       <c r="O19">
         <v>0</v>
       </c>
-      <c r="P19" t="str">
-        <v>6/12</v>
+      <c r="P19" t="s">
+        <v>22</v>
       </c>
       <c r="Q19">
+        <f t="shared" si="0"/>
         <v>120000</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
-      <c r="B20" t="str">
-        <v>Jusuf Habibi Muchtar</v>
-      </c>
-      <c r="C20" t="str">
-        <v>-</v>
+      <c r="B20" t="s">
+        <v>47</v>
+      </c>
+      <c r="C20" t="s">
+        <v>24</v>
       </c>
       <c r="D20">
         <v>0</v>
@@ -1453,22 +1771,23 @@
       <c r="O20">
         <v>0</v>
       </c>
-      <c r="P20" t="str">
-        <v>0/12</v>
+      <c r="P20" t="s">
+        <v>26</v>
       </c>
       <c r="Q20">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
-      <c r="B21" t="str">
-        <v>Khaerul Basyar Rukmana</v>
-      </c>
-      <c r="C21" t="str">
-        <v>085710401552</v>
+      <c r="B21" t="s">
+        <v>48</v>
+      </c>
+      <c r="C21" t="s">
+        <v>49</v>
       </c>
       <c r="D21">
         <v>20000</v>
@@ -1506,22 +1825,23 @@
       <c r="O21">
         <v>0</v>
       </c>
-      <c r="P21" t="str">
-        <v>2/12</v>
+      <c r="P21" t="s">
+        <v>19</v>
       </c>
       <c r="Q21">
+        <f t="shared" si="0"/>
         <v>40000</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
-      <c r="B22" t="str">
-        <v>Khairunnisa Dwi Kurniawan</v>
-      </c>
-      <c r="C22" t="str">
-        <v>-</v>
+      <c r="B22" t="s">
+        <v>50</v>
+      </c>
+      <c r="C22" t="s">
+        <v>24</v>
       </c>
       <c r="D22">
         <v>20000</v>
@@ -1559,22 +1879,23 @@
       <c r="O22">
         <v>0</v>
       </c>
-      <c r="P22" t="str">
-        <v>5/12</v>
+      <c r="P22" t="s">
+        <v>41</v>
       </c>
       <c r="Q22">
+        <f t="shared" si="0"/>
         <v>100000</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
-      <c r="B23" t="str">
-        <v>Kim Reynand Andah Pranaja</v>
-      </c>
-      <c r="C23" t="str">
-        <v>085117070159</v>
+      <c r="B23" t="s">
+        <v>51</v>
+      </c>
+      <c r="C23" t="s">
+        <v>52</v>
       </c>
       <c r="D23">
         <v>20000</v>
@@ -1612,22 +1933,23 @@
       <c r="O23">
         <v>0</v>
       </c>
-      <c r="P23" t="str">
-        <v>6/12</v>
+      <c r="P23" t="s">
+        <v>22</v>
       </c>
       <c r="Q23">
+        <f t="shared" si="0"/>
         <v>120000</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
-      <c r="B24" t="str">
-        <v>Lutfi Khoirul Nur Ramadhan</v>
-      </c>
-      <c r="C24" t="str">
-        <v>081283016613</v>
+      <c r="B24" t="s">
+        <v>53</v>
+      </c>
+      <c r="C24" t="s">
+        <v>54</v>
       </c>
       <c r="D24">
         <v>20000</v>
@@ -1665,22 +1987,23 @@
       <c r="O24">
         <v>20000</v>
       </c>
-      <c r="P24" t="str">
-        <v>12/12</v>
+      <c r="P24" t="s">
+        <v>32</v>
       </c>
       <c r="Q24">
+        <f t="shared" si="0"/>
         <v>240000</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
-      <c r="B25" t="str">
-        <v>Marco Alejandro Mendoza Retno</v>
-      </c>
-      <c r="C25" t="str">
-        <v>081808251119</v>
+      <c r="B25" t="s">
+        <v>55</v>
+      </c>
+      <c r="C25" t="s">
+        <v>56</v>
       </c>
       <c r="D25">
         <v>20000</v>
@@ -1718,22 +2041,23 @@
       <c r="O25">
         <v>0</v>
       </c>
-      <c r="P25" t="str">
-        <v>6/12</v>
+      <c r="P25" t="s">
+        <v>22</v>
       </c>
       <c r="Q25">
+        <f t="shared" si="0"/>
         <v>120000</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
-      <c r="B26" t="str">
-        <v>Maryam Audra Milly</v>
-      </c>
-      <c r="C26" t="str">
-        <v>085176651200</v>
+      <c r="B26" t="s">
+        <v>57</v>
+      </c>
+      <c r="C26" t="s">
+        <v>58</v>
       </c>
       <c r="D26">
         <v>20000</v>
@@ -1771,22 +2095,23 @@
       <c r="O26">
         <v>0</v>
       </c>
-      <c r="P26" t="str">
-        <v>2/12</v>
+      <c r="P26" t="s">
+        <v>19</v>
       </c>
       <c r="Q26">
+        <f t="shared" si="0"/>
         <v>40000</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
-      <c r="B27" t="str">
-        <v>Muhammad Danish Ali Haidari</v>
-      </c>
-      <c r="C27" t="str">
-        <v>-</v>
+      <c r="B27" t="s">
+        <v>59</v>
+      </c>
+      <c r="C27" t="s">
+        <v>24</v>
       </c>
       <c r="D27">
         <v>0</v>
@@ -1824,22 +2149,23 @@
       <c r="O27">
         <v>0</v>
       </c>
-      <c r="P27" t="str">
-        <v>0/12</v>
+      <c r="P27" t="s">
+        <v>26</v>
       </c>
       <c r="Q27">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
-      <c r="B28" t="str">
-        <v>Muhammad Raja El Firdaus</v>
-      </c>
-      <c r="C28" t="str">
-        <v>087745525749</v>
+      <c r="B28" t="s">
+        <v>60</v>
+      </c>
+      <c r="C28" t="s">
+        <v>61</v>
       </c>
       <c r="D28">
         <v>20000</v>
@@ -1877,22 +2203,23 @@
       <c r="O28">
         <v>0</v>
       </c>
-      <c r="P28" t="str">
-        <v>6/12</v>
+      <c r="P28" t="s">
+        <v>22</v>
       </c>
       <c r="Q28">
+        <f t="shared" si="0"/>
         <v>120000</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
-      <c r="B29" t="str">
-        <v>Muhammad Rifat Ramadhan</v>
-      </c>
-      <c r="C29" t="str">
-        <v>081212855837</v>
+      <c r="B29" t="s">
+        <v>62</v>
+      </c>
+      <c r="C29" t="s">
+        <v>63</v>
       </c>
       <c r="D29">
         <v>20000</v>
@@ -1930,75 +2257,77 @@
       <c r="O29">
         <v>0</v>
       </c>
-      <c r="P29" t="str">
-        <v>3/12</v>
+      <c r="P29" t="s">
+        <v>37</v>
       </c>
       <c r="Q29">
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
-      <c r="B30" t="str">
-        <v>Muhammad Zlatan Alkhalifi</v>
-      </c>
-      <c r="C30" t="str">
-        <v>081216100160</v>
+      <c r="B30" t="s">
+        <v>64</v>
+      </c>
+      <c r="C30" t="s">
+        <v>65</v>
       </c>
       <c r="D30">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="E30">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="F30">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="G30">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="H30">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="I30">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="J30">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="K30">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="L30">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="M30">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="N30">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="O30">
-        <v>0</v>
-      </c>
-      <c r="P30" t="str">
-        <v>0/12</v>
+        <v>20000</v>
+      </c>
+      <c r="P30" t="s">
+        <v>26</v>
       </c>
       <c r="Q30">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
+        <f t="shared" si="0"/>
+        <v>240000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
-      <c r="B31" t="str">
-        <v>Nathaniel Raphael</v>
-      </c>
-      <c r="C31" t="str">
-        <v>-</v>
+      <c r="B31" t="s">
+        <v>66</v>
+      </c>
+      <c r="C31" t="s">
+        <v>24</v>
       </c>
       <c r="D31">
         <v>20000</v>
@@ -2036,22 +2365,23 @@
       <c r="O31">
         <v>0</v>
       </c>
-      <c r="P31" t="str">
-        <v>3/12</v>
+      <c r="P31" t="s">
+        <v>37</v>
       </c>
       <c r="Q31">
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
-      <c r="B32" t="str">
-        <v>Naura Alvy Zahya</v>
-      </c>
-      <c r="C32" t="str">
-        <v>081291890142</v>
+      <c r="B32" t="s">
+        <v>67</v>
+      </c>
+      <c r="C32" t="s">
+        <v>68</v>
       </c>
       <c r="D32">
         <v>20000</v>
@@ -2089,22 +2419,23 @@
       <c r="O32">
         <v>20000</v>
       </c>
-      <c r="P32" t="str">
-        <v>12/12</v>
+      <c r="P32" t="s">
+        <v>32</v>
       </c>
       <c r="Q32">
+        <f t="shared" si="0"/>
         <v>240000</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
-      <c r="B33" t="str">
-        <v>Queenzha Aqila</v>
-      </c>
-      <c r="C33" t="str">
-        <v>081288071004</v>
+      <c r="B33" t="s">
+        <v>69</v>
+      </c>
+      <c r="C33" t="s">
+        <v>70</v>
       </c>
       <c r="D33">
         <v>20000</v>
@@ -2142,40 +2473,41 @@
       <c r="O33">
         <v>20000</v>
       </c>
-      <c r="P33" t="str">
-        <v>12/12</v>
+      <c r="P33" t="s">
+        <v>32</v>
       </c>
       <c r="Q33">
+        <f t="shared" si="0"/>
         <v>240000</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
-      <c r="B34" t="str">
-        <v>Satya Akbar Putra</v>
-      </c>
-      <c r="C34" t="str">
-        <v>-</v>
+      <c r="B34" t="s">
+        <v>71</v>
+      </c>
+      <c r="C34" t="s">
+        <v>24</v>
       </c>
       <c r="D34">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="E34">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="F34">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="G34">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="H34">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="I34">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="J34">
         <v>0</v>
@@ -2195,22 +2527,23 @@
       <c r="O34">
         <v>0</v>
       </c>
-      <c r="P34" t="str">
-        <v>0/12</v>
+      <c r="P34" t="s">
+        <v>26</v>
       </c>
       <c r="Q34">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
+        <f t="shared" si="0"/>
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
-      <c r="B35" t="str">
-        <v>Syafhia Nazruliza</v>
-      </c>
-      <c r="C35" t="str">
-        <v>-</v>
+      <c r="B35" t="s">
+        <v>72</v>
+      </c>
+      <c r="C35" t="s">
+        <v>24</v>
       </c>
       <c r="D35">
         <v>0</v>
@@ -2248,22 +2581,23 @@
       <c r="O35">
         <v>0</v>
       </c>
-      <c r="P35" t="str">
-        <v>0/12</v>
+      <c r="P35" t="s">
+        <v>26</v>
       </c>
       <c r="Q35">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
-      <c r="B36" t="str">
-        <v>Viola Callista Donita</v>
-      </c>
-      <c r="C36" t="str">
-        <v>08111742629</v>
+      <c r="B36" t="s">
+        <v>73</v>
+      </c>
+      <c r="C36" t="s">
+        <v>36</v>
       </c>
       <c r="D36">
         <v>20000</v>
@@ -2301,180 +2635,195 @@
       <c r="O36">
         <v>0</v>
       </c>
-      <c r="P36" t="str">
-        <v>3/12</v>
+      <c r="P36" t="s">
+        <v>37</v>
       </c>
       <c r="Q36">
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
     </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="Q37">
+        <f>SUM(Q2:Q36)</f>
+        <v>3660000</v>
+      </c>
+    </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q36"/>
+    <ignoredError sqref="A1:Q1 A7:P7 A6:C6 J6:P6 A14:P16 A13:C13 I13:P13 A3:P5 A2:P2 A18:P29 A17:C17 F17:P17 A31:P33 A30:C30 P30 A12:C12 I12:P12 A9:P11 A8:C8 I8:P8 A35:P36 A34:C34 J34:P34" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="63.5" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>No</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Tanggal</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Kategori</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Uraian Keperluan</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Nominal (Rp)</v>
-      </c>
-    </row>
-    <row r="2">
+    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="str">
-        <v>2026-08-10</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Keperluan Kelas</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Keperluan &amp; Kegiatan Kelas 5A</v>
+      <c r="B2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D2" t="s">
+        <v>80</v>
       </c>
       <c r="E2">
-        <v>43000</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>48735</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="str">
-        <v>2026-08-04</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Lain-lain</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Tissue 2 Ply A Basics 600gram 2pcs</v>
+      <c r="B3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D3" t="s">
+        <v>81</v>
       </c>
       <c r="E3">
-        <v>48735</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>58600</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" t="str">
-        <v>2026-08-04</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Lain-lain</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Stella Aerosol Balinese Jasmine Sensation Pengharum Ruangan 350ml 2pcs</v>
+      <c r="B4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" t="s">
+        <v>79</v>
+      </c>
+      <c r="D4" t="s">
+        <v>83</v>
       </c>
       <c r="E4">
-        <v>58600</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>44000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" t="str">
-        <v>2026-07-31</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Lain-lain</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Air galon 2 @22000</v>
+      <c r="B5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D5" t="s">
+        <v>84</v>
       </c>
       <c r="E5">
-        <v>44000</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" t="str">
-        <v>2026-07-31</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Lain-lain</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Tisue</v>
+      <c r="B6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C6" t="s">
+        <v>85</v>
+      </c>
+      <c r="D6" t="s">
+        <v>86</v>
       </c>
       <c r="E6">
-        <v>35000</v>
-      </c>
-    </row>
-    <row r="7">
+        <v>17500</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" t="str">
-        <v>2026-07-31</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Fotokopi &amp; Cetak Soal</v>
-      </c>
-      <c r="D7" t="str">
-        <v>FC jadwal 35 @500</v>
+      <c r="B7" t="s">
+        <v>82</v>
+      </c>
+      <c r="C7" t="s">
+        <v>85</v>
+      </c>
+      <c r="D7" t="s">
+        <v>87</v>
       </c>
       <c r="E7">
-        <v>17500</v>
-      </c>
-    </row>
-    <row r="8">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" t="str">
-        <v>2026-07-31</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Fotokopi &amp; Cetak Soal</v>
-      </c>
-      <c r="D8" t="str">
-        <v>LKPD MPLS 20 @500</v>
+      <c r="B8" t="s">
+        <v>82</v>
+      </c>
+      <c r="C8" t="s">
+        <v>85</v>
+      </c>
+      <c r="D8" t="s">
+        <v>88</v>
       </c>
       <c r="E8">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="9">
+        <v>17500</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" t="str">
-        <v>2026-07-31</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Fotokopi &amp; Cetak Soal</v>
-      </c>
-      <c r="D9" t="str">
-        <v>LKPD Wali kelas 35 @500</v>
+      <c r="B9" s="1">
+        <v>46246</v>
+      </c>
+      <c r="C9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D9" t="s">
+        <v>89</v>
       </c>
       <c r="E9">
-        <v>17500</v>
+        <v>43000</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+    <ignoredError sqref="A1:E8" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>